<commit_message>
for "Waiting for OLE action in another program to complete."
</commit_message>
<xml_diff>
--- a/out/aaa.xlsx
+++ b/out/aaa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitwork\CreateTableOfContentsExcelUsingSheetNames\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC2BE178-5E3F-4EFA-A20E-08867BEAC4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3A9B523-4513-4311-A776-4F6A2DF8C108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="23840" windowHeight="12700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1760" yWindow="3300" windowWidth="23840" windowHeight="12700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="２ページ" sheetId="4" r:id="rId1"/>

</xml_diff>